<commit_message>
Rebuild the Max Mara workbook so Excel opens it normally.
The previous file opened in page-break preview with a frozen-pane selection Excel treats as damaged.

Co-authored-by: leaf405-wq <leaf405-wq@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/store-ops/docs/MaxMara_Deliverables_v1.xlsx
+++ b/store-ops/docs/MaxMara_Deliverables_v1.xlsx
@@ -520,7 +520,7 @@
   <sheetPr>
     <tabColor rgb="008C3F1C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1598,7 +1598,7 @@
   <sheetPr>
     <tabColor rgb="008C3F1C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2282,7 +2282,7 @@
   <sheetPr>
     <tabColor rgb="008C3F1C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3134,7 +3134,7 @@
   <sheetPr>
     <tabColor rgb="008C3F1C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4277,7 +4277,7 @@
   <sheetPr>
     <tabColor rgb="008C3F1C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4649,7 +4649,7 @@
   <sheetPr>
     <tabColor rgb="008C3F1C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>

</xml_diff>